<commit_message>
Update batting and bowling
</commit_message>
<xml_diff>
--- a/data/cricket_stats.xlsx
+++ b/data/cricket_stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Desktop\My cricket dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3710B51E-2190-485E-933F-9FB87551436A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{570F446B-C32B-4A51-9E68-1E32004B866C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{E6DD8058-5BE6-400D-BF11-B271C0BD4B9B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E6DD8058-5BE6-400D-BF11-B271C0BD4B9B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="58">
   <si>
     <t>Date</t>
   </si>
@@ -74,12 +74,6 @@
     <t>HnH</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Stump</t>
-  </si>
-  <si>
     <t>Runout</t>
   </si>
   <si>
@@ -105,13 +99,205 @@
   </si>
   <si>
     <t>Practice matches</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Kaluthara PCC </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(20)</t>
+    </r>
+  </si>
+  <si>
+    <t>Mas Active</t>
+  </si>
+  <si>
+    <t>Panagoda CC</t>
+  </si>
+  <si>
+    <t>Horana Royal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Western Phoenix </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">VSIS   </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(25)</t>
+    </r>
+  </si>
+  <si>
+    <t>Mayans</t>
+  </si>
+  <si>
+    <t>KTC</t>
+  </si>
+  <si>
+    <t>Capricorn CC</t>
+  </si>
+  <si>
+    <t>Mt Lavinia CC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Old Centralians </t>
+  </si>
+  <si>
+    <t>Katubedda SC</t>
+  </si>
+  <si>
+    <t>Eagles CC</t>
+  </si>
+  <si>
+    <t>Uni of Kelaniya</t>
+  </si>
+  <si>
+    <t>Ruhuna University</t>
+  </si>
+  <si>
+    <t>Others</t>
+  </si>
+  <si>
+    <t>Division 3</t>
+  </si>
+  <si>
+    <t>Inter Uni</t>
+  </si>
+  <si>
+    <t>LBW</t>
+  </si>
+  <si>
+    <t>Bowled</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>Ananda CC</t>
+  </si>
+  <si>
+    <t>Catamarans CC</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">HnH  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(25)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">HnH </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(15)</t>
+    </r>
+  </si>
+  <si>
+    <t>Mt Lavinia</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Old Rajians </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(20)</t>
+    </r>
+  </si>
+  <si>
+    <t>Mohras CC</t>
+  </si>
+  <si>
+    <t>Lankan CC</t>
+  </si>
+  <si>
+    <t>NWSC</t>
+  </si>
+  <si>
+    <r>
+      <t>HnH</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(20)</t>
+    </r>
+  </si>
+  <si>
+    <t>Liberty CC B</t>
+  </si>
+  <si>
+    <t>Memon SC</t>
+  </si>
+  <si>
+    <t>Caught</t>
+  </si>
+  <si>
+    <t>Hit Wkt</t>
+  </si>
+  <si>
+    <t>Caught B</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,16 +305,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -136,12 +342,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -476,183 +715,1344 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E054A30-9585-4C99-98B9-8637B289CECB}">
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:R40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="21.28515625" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="1"/>
+    <col min="3" max="3" width="21.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18" style="1" customWidth="1"/>
+    <col min="5" max="12" width="9.140625" style="1"/>
+    <col min="13" max="13" width="9.42578125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="13.28515625" style="1" customWidth="1"/>
+    <col min="15" max="18" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+    <row r="1" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M1" t="s">
+      <c r="L1" s="4"/>
+      <c r="M1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="O1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B2" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>2</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K2" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B3" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="1">
+        <v>5</v>
+      </c>
+      <c r="F3" s="1">
+        <v>12</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B4" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="P1" t="s">
+      <c r="D4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2">
+        <v>2</v>
+      </c>
+      <c r="N4" s="1">
+        <v>6</v>
+      </c>
+      <c r="O4" s="1">
+        <v>0</v>
+      </c>
+      <c r="P4" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B5" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B2">
+      <c r="D5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="1">
+        <v>1</v>
+      </c>
+      <c r="M5" s="2">
+        <v>8</v>
+      </c>
+      <c r="N5" s="1">
+        <v>21</v>
+      </c>
+      <c r="O5" s="1">
+        <v>1</v>
+      </c>
+      <c r="P5" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B6" s="1">
         <v>2024</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6" s="1">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2">
+        <v>3</v>
+      </c>
+      <c r="N6" s="1">
+        <v>16</v>
+      </c>
+      <c r="O6" s="1">
+        <v>0</v>
+      </c>
+      <c r="P6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
+      <c r="K7" s="1">
         <v>2</v>
       </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="M7" s="2">
+        <v>7</v>
+      </c>
+      <c r="N7" s="1">
+        <v>52</v>
+      </c>
+      <c r="O7" s="1">
+        <v>0</v>
+      </c>
+      <c r="P7" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B8" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2">
+        <v>4</v>
+      </c>
+      <c r="N8" s="1">
+        <v>31</v>
+      </c>
+      <c r="O8" s="1">
+        <v>0</v>
+      </c>
+      <c r="P8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B9" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K9" s="1">
+        <v>0</v>
+      </c>
+      <c r="M9" s="2">
+        <v>5</v>
+      </c>
+      <c r="N9" s="1">
+        <v>40</v>
+      </c>
+      <c r="O9" s="1">
+        <v>0</v>
+      </c>
+      <c r="P9" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B10" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="1">
+        <v>11</v>
+      </c>
+      <c r="F10" s="1">
+        <v>48</v>
+      </c>
+      <c r="G10" s="1">
+        <v>0</v>
+      </c>
+      <c r="H10" s="1">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K10" s="1">
+        <v>0</v>
+      </c>
+      <c r="M10" s="2">
+        <v>7</v>
+      </c>
+      <c r="N10" s="1">
+        <v>34</v>
+      </c>
+      <c r="O10" s="1">
+        <v>0</v>
+      </c>
+      <c r="P10" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B11" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="1">
+        <v>6</v>
+      </c>
+      <c r="F11" s="1">
+        <v>17</v>
+      </c>
+      <c r="G11" s="1">
+        <v>0</v>
+      </c>
+      <c r="H11" s="1">
+        <v>0</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K11" s="1">
+        <v>0</v>
+      </c>
+      <c r="M11" s="2">
+        <v>6</v>
+      </c>
+      <c r="N11" s="1">
+        <v>35</v>
+      </c>
+      <c r="O11" s="1">
+        <v>0</v>
+      </c>
+      <c r="P11" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B12" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="1">
+        <v>7</v>
+      </c>
+      <c r="F12" s="1">
+        <v>27</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K12" s="1">
+        <v>1</v>
+      </c>
+      <c r="M12" s="2">
+        <v>7.2</v>
+      </c>
+      <c r="N12" s="1">
+        <v>28</v>
+      </c>
+      <c r="O12" s="1">
+        <v>0</v>
+      </c>
+      <c r="P12" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B13" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K13" s="1">
+        <v>0</v>
+      </c>
+      <c r="M13" s="2">
+        <v>10</v>
+      </c>
+      <c r="N13" s="1">
+        <v>52</v>
+      </c>
+      <c r="O13" s="1">
+        <v>0</v>
+      </c>
+      <c r="P13" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B14" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K14" s="1">
+        <v>1</v>
+      </c>
+      <c r="M14" s="2">
+        <v>9.1</v>
+      </c>
+      <c r="N14" s="1">
+        <v>14</v>
+      </c>
+      <c r="O14" s="1">
+        <v>2</v>
+      </c>
+      <c r="P14" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B15" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1</v>
+      </c>
+      <c r="M15" s="2">
+        <v>5</v>
+      </c>
+      <c r="N15" s="1">
+        <v>32</v>
+      </c>
+      <c r="O15" s="1">
+        <v>0</v>
+      </c>
+      <c r="P15" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B16" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K16" s="1">
+        <v>0</v>
+      </c>
+      <c r="M16" s="2">
+        <v>10</v>
+      </c>
+      <c r="N16" s="1">
+        <v>55</v>
+      </c>
+      <c r="O16" s="1">
+        <v>0</v>
+      </c>
+      <c r="P16" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B17" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K17" s="1">
+        <v>0</v>
+      </c>
+      <c r="M17" s="2">
+        <v>8</v>
+      </c>
+      <c r="N17" s="1">
+        <v>35</v>
+      </c>
+      <c r="O17" s="1">
+        <v>0</v>
+      </c>
+      <c r="P17" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B18" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K18" s="1">
+        <v>0</v>
+      </c>
+      <c r="M18" s="2">
+        <v>6</v>
+      </c>
+      <c r="N18" s="1">
+        <v>11</v>
+      </c>
+      <c r="O18" s="1">
+        <v>1</v>
+      </c>
+      <c r="P18" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B19" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K19" s="1">
+        <v>0</v>
+      </c>
+      <c r="M19" s="2">
+        <v>3</v>
+      </c>
+      <c r="N19" s="1">
+        <v>20</v>
+      </c>
+      <c r="O19" s="1">
+        <v>0</v>
+      </c>
+      <c r="P19" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B20" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="1">
+        <v>4</v>
+      </c>
+      <c r="F20" s="1">
         <v>12</v>
       </c>
-      <c r="J2" t="s">
+      <c r="G20" s="1">
+        <v>0</v>
+      </c>
+      <c r="H20" s="1">
+        <v>0</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="K20" s="1">
+        <v>0</v>
+      </c>
+      <c r="M20" s="2"/>
+    </row>
+    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B21" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" s="1">
+        <v>0</v>
+      </c>
+      <c r="F21" s="1">
+        <v>1</v>
+      </c>
+      <c r="G21" s="1">
+        <v>0</v>
+      </c>
+      <c r="H21" s="1">
+        <v>0</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K21" s="1">
+        <v>0</v>
+      </c>
+      <c r="M21" s="2">
+        <v>3</v>
+      </c>
+      <c r="N21" s="1">
+        <v>18</v>
+      </c>
+      <c r="O21" s="1">
+        <v>0</v>
+      </c>
+      <c r="P21" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B22" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" s="1">
+        <v>10</v>
+      </c>
+      <c r="F22" s="1">
         <v>13</v>
       </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>3.2</v>
-      </c>
-      <c r="N2">
+      <c r="G22" s="1">
+        <v>1</v>
+      </c>
+      <c r="H22" s="1">
+        <v>0</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="K22" s="1">
+        <v>0</v>
+      </c>
+      <c r="M22" s="2">
+        <v>9</v>
+      </c>
+      <c r="N22" s="1">
+        <v>34</v>
+      </c>
+      <c r="O22" s="1">
+        <v>0</v>
+      </c>
+      <c r="P22" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B23" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K23" s="1">
+        <v>0</v>
+      </c>
+      <c r="M23" s="2">
+        <v>3</v>
+      </c>
+      <c r="N23" s="1">
+        <v>5</v>
+      </c>
+      <c r="O23" s="1">
+        <v>1</v>
+      </c>
+      <c r="P23" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B24" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K24" s="1">
+        <v>0</v>
+      </c>
+      <c r="M24" s="2">
+        <v>5</v>
+      </c>
+      <c r="N24" s="1">
+        <v>20</v>
+      </c>
+      <c r="O24" s="1">
+        <v>0</v>
+      </c>
+      <c r="P24" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B25" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" s="1">
+        <v>1</v>
+      </c>
+      <c r="F25" s="1">
+        <v>4</v>
+      </c>
+      <c r="G25" s="1">
+        <v>0</v>
+      </c>
+      <c r="H25" s="1">
+        <v>0</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K25" s="1">
+        <v>0</v>
+      </c>
+      <c r="M25" s="2">
+        <v>4</v>
+      </c>
+      <c r="N25" s="1">
+        <v>14</v>
+      </c>
+      <c r="O25" s="1">
+        <v>1</v>
+      </c>
+      <c r="P25" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B26" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K26" s="1">
+        <v>0</v>
+      </c>
+      <c r="M26" s="2">
+        <v>7</v>
+      </c>
+      <c r="N26" s="1">
+        <v>17</v>
+      </c>
+      <c r="O26" s="1">
+        <v>1</v>
+      </c>
+      <c r="P26" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B27" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K27" s="1">
+        <v>1</v>
+      </c>
+      <c r="M27" s="2">
+        <v>3</v>
+      </c>
+      <c r="N27" s="1">
+        <v>13</v>
+      </c>
+      <c r="O27" s="1">
+        <v>0</v>
+      </c>
+      <c r="P27" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B28" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" s="1">
+        <v>22</v>
+      </c>
+      <c r="F28" s="1">
+        <v>33</v>
+      </c>
+      <c r="G28" s="1">
+        <v>1</v>
+      </c>
+      <c r="H28" s="1">
+        <v>0</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="K28" s="1">
+        <v>0</v>
+      </c>
+      <c r="M28" s="2">
+        <v>5</v>
+      </c>
+      <c r="N28" s="1">
         <v>12</v>
       </c>
-      <c r="O2">
+      <c r="O28" s="1">
+        <v>1</v>
+      </c>
+      <c r="P28" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B29" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" s="1">
+        <v>6</v>
+      </c>
+      <c r="F29" s="1">
+        <v>6</v>
+      </c>
+      <c r="G29" s="1">
+        <v>0</v>
+      </c>
+      <c r="H29" s="1">
+        <v>0</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K29" s="1">
+        <v>0</v>
+      </c>
+      <c r="M29" s="2">
+        <v>3</v>
+      </c>
+      <c r="N29" s="1">
+        <v>28</v>
+      </c>
+      <c r="O29" s="1">
+        <v>0</v>
+      </c>
+      <c r="P29" s="1">
         <v>2</v>
       </c>
-      <c r="P2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B3">
-        <v>2024</v>
-      </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B30" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K30" s="1">
+        <v>0</v>
+      </c>
+      <c r="M30" s="2">
+        <v>6</v>
+      </c>
+      <c r="N30" s="1">
+        <v>26</v>
+      </c>
+      <c r="O30" s="1">
+        <v>0</v>
+      </c>
+      <c r="P30" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B31" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E31" s="1">
+        <v>15</v>
+      </c>
+      <c r="F31" s="1">
+        <v>26</v>
+      </c>
+      <c r="G31" s="1">
+        <v>1</v>
+      </c>
+      <c r="H31" s="1">
+        <v>0</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="K31" s="1">
+        <v>0</v>
+      </c>
+      <c r="M31" s="2">
+        <v>6</v>
+      </c>
+      <c r="N31" s="1">
+        <v>15</v>
+      </c>
+      <c r="O31" s="1">
+        <v>1</v>
+      </c>
+      <c r="P31" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B32" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K32" s="1">
+        <v>0</v>
+      </c>
+      <c r="M32" s="2">
+        <v>2</v>
+      </c>
+      <c r="N32" s="1">
+        <v>12</v>
+      </c>
+      <c r="O32" s="1">
+        <v>0</v>
+      </c>
+      <c r="P32" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B33" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K33" s="1">
+        <v>1</v>
+      </c>
+      <c r="M33" s="2">
+        <v>4</v>
+      </c>
+      <c r="N33" s="1">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
+      <c r="O33" s="1">
+        <v>0</v>
+      </c>
+      <c r="P33" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B34" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K34" s="1">
+        <v>0</v>
+      </c>
+      <c r="M34" s="2">
+        <v>8.4</v>
+      </c>
+      <c r="N34" s="1">
+        <v>24</v>
+      </c>
+      <c r="O34" s="1">
+        <v>3</v>
+      </c>
+      <c r="P34" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B35" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E35" s="1">
+        <v>4</v>
+      </c>
+      <c r="F35" s="1">
+        <v>7</v>
+      </c>
+      <c r="G35" s="1">
+        <v>0</v>
+      </c>
+      <c r="H35" s="1">
+        <v>0</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="K35" s="1">
+        <v>0</v>
+      </c>
+      <c r="M35" s="2">
+        <v>5</v>
+      </c>
+      <c r="N35" s="1">
+        <v>17</v>
+      </c>
+      <c r="O35" s="1">
+        <v>1</v>
+      </c>
+      <c r="P35" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B36" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E36" s="1">
         <v>11</v>
       </c>
-      <c r="E3">
-        <v>5</v>
-      </c>
-      <c r="F3">
-        <v>12</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>2.5</v>
-      </c>
-      <c r="N3">
+      <c r="F36" s="1">
+        <v>8</v>
+      </c>
+      <c r="G36" s="1">
+        <v>1</v>
+      </c>
+      <c r="H36" s="1">
+        <v>0</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="K36" s="1">
+        <v>1</v>
+      </c>
+      <c r="M36" s="1">
         <v>10</v>
       </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
+      <c r="N36" s="1">
+        <v>29</v>
+      </c>
+      <c r="O36" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B4">
-        <v>2024</v>
-      </c>
-      <c r="C4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B5">
-        <v>2024</v>
-      </c>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B6">
-        <v>2024</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="P36" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B37" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" s="1">
+        <v>17</v>
+      </c>
+      <c r="F37" s="1">
+        <v>27</v>
+      </c>
+      <c r="G37" s="1">
+        <v>2</v>
+      </c>
+      <c r="H37" s="1">
+        <v>0</v>
+      </c>
+      <c r="I37" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D6" t="s">
-        <v>22</v>
+      <c r="J37" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K37" s="1">
+        <v>0</v>
+      </c>
+      <c r="M37" s="1">
+        <v>4</v>
+      </c>
+      <c r="N37" s="1">
+        <v>16</v>
+      </c>
+      <c r="O37" s="1">
+        <v>1</v>
+      </c>
+      <c r="P37" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B38" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K38" s="1">
+        <v>0</v>
+      </c>
+      <c r="M38" s="1">
+        <v>9</v>
+      </c>
+      <c r="N38" s="1">
+        <v>21</v>
+      </c>
+      <c r="O38" s="1">
+        <v>1</v>
+      </c>
+      <c r="P38" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B39" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E39" s="1">
+        <v>4</v>
+      </c>
+      <c r="F39" s="1">
+        <v>7</v>
+      </c>
+      <c r="G39" s="1">
+        <v>0</v>
+      </c>
+      <c r="H39" s="1">
+        <v>0</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K39" s="1">
+        <v>0</v>
+      </c>
+      <c r="M39" s="1">
+        <v>4</v>
+      </c>
+      <c r="N39" s="1">
+        <v>18</v>
+      </c>
+      <c r="O39" s="1">
+        <v>0</v>
+      </c>
+      <c r="P39" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B40" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" s="1">
+        <v>30</v>
+      </c>
+      <c r="F40" s="1">
+        <v>49</v>
+      </c>
+      <c r="G40" s="1">
+        <v>3</v>
+      </c>
+      <c r="H40" s="1">
+        <v>0</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K40" s="1">
+        <v>0</v>
+      </c>
+      <c r="M40" s="1">
+        <v>8</v>
+      </c>
+      <c r="N40" s="1">
+        <v>41</v>
+      </c>
+      <c r="O40" s="1">
+        <v>0</v>
+      </c>
+      <c r="P40" s="1">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -808,20 +2208,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="e9fca74d-1c08-4535-9786-05f793b2565f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="e9fca74d-1c08-4535-9786-05f793b2565f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -843,6 +2243,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{384823D1-2E94-403E-BF12-2D5DE0378A7F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E325A0B-8866-4BFA-81B8-B75F7233D469}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -856,12 +2264,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{384823D1-2E94-403E-BF12-2D5DE0378A7F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>